<commit_message>
Add cards-category, columns-diptych, hero-banner blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (10):
- blocks/cards-category/cards-category.css
- blocks/columns-diptych/columns-diptych.css
- blocks/hero-banner/hero-banner.css
- blocks/hero-banner/hero-banner.js
- tools/importer/import-homepage.bundle.js
- tools/importer/import-homepage.js
- tools/importer/page-templates.json
- tools/importer/parsers/hero-banner.js
- tools/importer/reports/import-homepage.report.xlsx
- tools/importer/reports/index.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero-banner","hero-banner","hero-banner","hero-banner","hero-banner","hero-banner","carousel-product","carousel-product","columns-diptych","columns-diptych","columns-diptych","columns-diptych","cards-category","embed-social","cards-feature","cards-service"]</t>
+    <t>["hero-banner","hero-banner","hero-banner","carousel-product","carousel-product","columns-diptych","columns-diptych","cards-category","embed-social","cards-feature","cards-service"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-03-25T16:16:18.483Z</t>
+    <t>2026-03-25T19:19:02.259Z</t>
   </si>
   <si>
     <t>Faherty Brand - Official Site - Free Shipping on Orders $150+</t>

</xml_diff>